<commit_message>
Add Tennessee hub and regroup geography navigation.
Split East TN / statewide cases onto tennessee.html, keep Crossville focused on local action, brand the dossier PDF/Excel exports to match the site, and put Crossville · Tennessee · National beside each other in the top nav.
</commit_message>
<xml_diff>
--- a/docs/Flock_Municipal_Cancellations_Database.xlsx
+++ b/docs/Flock_Municipal_Cancellations_Database.xlsx
@@ -27,17 +27,28 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0392B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDF6F6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,13 +56,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,8 +450,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="48" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -493,2617 +542,3222 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Oshkosh</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>WI</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Rescinded</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2026-04-23</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>26</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Vendor misrepresentation (heat maps); Police chief trust failure; Public backlash</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Council approved a one-year renewal amid vocal public opposition, then unanimously rescinded within ~24 hours after Police Chief Dean Smith said Flock misrepresented heat-map tracking capability at the council meeting. Cameras powered off and bagged.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>https://www.postcrescent.com/story/news/local/oshkosh/2026/04/22/oshkosh-rescinds-flock-safety-contract-after-police-chief-raises-concerns/89745485007/</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>https://www.wbay.com/2026/04/23/oshkosh-council-rescinds-flock-camera-contract-after-false-statements/</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Hardware bagged while removal coordinated.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Verona</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>WI</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Non-renewal</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Public backlash; Loss of trust in vendor (not PD); Data-sharing / federal access fears</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Common Council voted not to renew; contract lapsed December. Officials and residents framed the decision as lack of public trust in Flock Safety. Cameras remained up for months; city covered them pending physical removal.</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>https://wisconsinexaminer.com/2026/02/02/verona-expected-to-begin-work-to-removing-flock-cameras/</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Physical removal lagged contract end; interim lens covers.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Staunton</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>2025-12-19</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Public backlash; Resident council testimony; CEO email conflicted with city values</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>After months of resident opposition at council (dozen speakers Dec. 11), Chief Jim Williams moved to cancel following a Flock CEO email the city said did not reflect Staunton’s values. Contract terminated Jan. 8, 2026; physical removal lagged.</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>https://augustafreepress.com/news/staunton-to-cancel-flock-safety-camera-contract-doesnt-agree-with-ideology-of-ceo/</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>https://www.whsv.com/2026/01/10/city-stauntons-contract-with-flock-safety-officially-terminated/</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Removal delayed; some cameras still up into Feb 2026 per News Leader.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Framingham</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Non-renewal</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Public backlash; Resident advocacy; Data sharing / oversight concerns</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Police will not renew after months of resident opposition. System access shut off at contract end; Flock to remove cameras. Follows Cambridge, Watertown, and Natick exits in Massachusetts.</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>https://www.boston.com/news/local-news/2026/06/25/framingham-police-will-not-renew-flock-safety-contract-after-months-of-resident-opposition/</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Advocates seeking assurance city will not replace with similar system.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Flagstaff</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>AZ</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Public backlash; Loss of community trust; Data-sharing concerns</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>After tightening sharing controls failed to restore trust, mayor and council ended the contract. NPR quotes Mayor Becky Daggett: technology would not be well received or continueable.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>https://www.npr.org/2026/02/17/nx-s1-5612825/flock-contracts-canceled-immigration-survillance-concerns</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Westland</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>MI</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Non-renewal</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Public backlash; Privacy / constitutional concerns; Outside agency / ICE access fears; Split council</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Police chief did not bring renewal to council after finding council deeply split. Council president cited privacy, corporate sharing, ICE access fears, and credited residents and advocacy groups for raising concerns.</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>https://www.clickondetroit.com/news/local/2026/07/10/westland-to-remove-flock-safety-license-plate-cameras-after-privacy-concerns/</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Verified local TV</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>Removal at contract expiration end of month.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Ithaca</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Public backlash; Sanctuary-city conflict; Third-party disclosure language; Outside agency access concerns</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Common Council ended the contract after activist campaign and protests outside city hall. Resolution cited sanctuary policies and documented outside-agency access without explicit local authorization.</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>https://www.wrvo.org/2026-03-05/ithaca-common-council-votes-to-end-contract-with-flock-safety</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Santa Cruz</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Out-of-state access; Immigration / sanctuary urgency; Public / grassroots pressure (Get the Flock Out)</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>Council voted 6-1 to terminate after out-of-state agencies accessed city data. Widely reported as first California city to end a Flock contract; grassroots organizing credited alongside immigration-enforcement urgency.</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>https://www.kqed.org/news/12069705/santa-cruz-the-first-in-california-to-terminate-its-contract-with-flock-safety</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>https://www.npr.org/2026/02/17/nx-s1-5612825/flock-contracts-canceled-immigration-survillance-concerns</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>South Portland</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>2026-06-11</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>7</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Public backlash; Privacy / constitutional concerns</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Council workshop directed end of Flock use after strong community backlash. All seven cameras removed by June 22, 2026; no active South Portland Flock account.</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>https://www.southportland.gov/m/NewsFlash/home/detail/550</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>https://www.pressherald.com/2026/07/01/south-portlands-flock-cameras-have-been-removed/</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Verified local/primary</t>
         </is>
       </c>
+      <c r="N10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Denver</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>CO</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Expired</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>2026-03-31</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>110</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Public backlash; Privacy concerns; Federal immigration data-sharing revelations</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>Largest reported single municipal removal by camera count: 110 intersection cameras decommissioned and removed when contract expired. City approved Axon replacement (~50 cams) with stricter controls.</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>https://www.9news.com/article/news/local/denver-removes-flock-license-plate-reader-cameras/73-eaf91d0a-3b90-45f5-8338-dbb9f79a8712</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>Verified local TV</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>Private/HOA Flock cameras remain; some pre-Flock city LPR gear unaffected.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-011</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>2025-06</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Public backlash; ICE data-sharing fears; Wrongful-arrest risk concerns</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>City canceled after organized community opposition. Later reporting that APD found ways to keep using Flock data through other agencies (loophole).</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>https://www.kut.org/crime-justice/2026-02-18/austin-ended-its-license-plate-reader-program-then-the-police-found-a-loophole</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>City contract end ≠ full network offline for police via partners.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>CAN-2025-012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Cambridge</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Unauthorized camera installs; Material breach of trust; Public scrutiny</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>City terminated after Flock installed cameras without city awareness/authorization; described as material breach of trust.</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>https://www.cambridgema.gov/news/2025/12/statementontheflocksafetyalprcontracttermination</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L13" s="3" t="inlineStr">
         <is>
           <t>https://www.boston.com/news/local-news/2025/12/11/cambridge-ends-contract-for-license-plate-cameras-after-breach-of-trust/</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>Verified local/primary</t>
         </is>
       </c>
+      <c r="N13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-013</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Mountain View</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Suspended</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>2026-02-03</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>30</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Unauthorized federal access (ATF; Air Force; GSA IG); Audit findings</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Disabled all ~30 cameras after audit showed federal agencies had accessed local data without authorization.</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>https://localnewsmatters.org/2026/03/03/mountain-view-terminates-license-plate-reader-contract-with-flock-safety/</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-014</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Oxnard</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Suspended</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>2026-02-27</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>19</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Vendor-enabled National Lookup vs California law; Out-of-state / federal queries; Public trust</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>OPD suspended 19 fixed Flock cameras after audit found nationwide query capability allowed out-of-state/federal agencies to include Oxnard data despite California-only settings.</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>https://www.oxnard.gov/pd-news/news-release-oxnard-police-department-suspends-use-of-flock-safety-automated-license-plate-readers-02-27-26</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>https://www.edhat.com/ventura/news/oxnard-police-suspend-flock-license-plate-readers-ventura-agencies-tighten-controls-after-out-of-state-access/</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>Verified local/primary</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>Suspension pending confidence in safeguards; not necessarily permanent cancel.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-015</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>South Pasadena</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>14</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Privacy concerns; Illegal sharing with federal immigration agents (regional reports)</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Council canceled contract for ~14 cameras after reports Southern California agencies shared Flock data with federal immigration agents.</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>https://laist.com/news/politics/south-pasadena-cancels-contract-with-flock-safety-citing-privacy-concerns</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-016</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Los Angeles Police Department</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Expired</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>138</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Privacy / civil liberties; Data ownership uncertainty; Federal access concerns</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>LAPD let three-year agreement expire (~138 pole cameras since 2023). Audit/reporting cited federal access and immigration-enforcement risk. Some outlets note possible renegotiation with stricter terms.</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>https://www.businessinsider.com/flock-safety-cameras-police-departments-lapd-2026-7</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr">
         <is>
           <t>https://www.cnet.com/news/privacy/los-angeles-lapd-flock-safety-surveillance-cameras-privacy/</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N17" s="3" t="inlineStr">
         <is>
           <t>May renegotiate; not necessarily a permanent ban.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-017</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Bloomington</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Expired</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Months-long evaluation; Oversight / legal considerations; Council oversight resolution context</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Mayor announced contract expired and city would not renew after evaluation with PD, legal, Flock, and community partners. Sharing narrowed during wind-down.</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>https://bloomington.in.gov/news/2026/04/15/6521</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Verified local/primary</t>
         </is>
       </c>
+      <c r="N18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-018</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Edmonds</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>19</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>New state ALPR law compliance; Retention / audit / disclosure liability; Staffing burden</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>Council unanimously authorized termination after procedural correction. Chief cited new state guardrails creating liability and records burdens.</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>https://www.heraldnet.com/2026/06/10/following-procedural-error-edmonds-unanimously-cancels-flock-contract/</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-019</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Evanston</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>2025-08</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>19</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Illinois SOS audit climate; Federal / CBP access concerns; Privacy</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Terminated ~19 cameras after Illinois audit climate showing CBP access to state plate networks. Later dispute: incomplete removal / alleged reinstall without permission; cease-and-desist reported.</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>https://www.eff.org/deeplinks/2026/02/get-flock-out-our-city</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>https://www.techtimes.com/articles/319317/20260629/flock-safety-crosses-100000-cameras-53-cities-cancel-over-unauthorized-federal-data-access.htm</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>Removal fight after cancel; confirm final hardware status.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>CAN-2025-020</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Oak Park</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>2025-08-05</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>8</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>Sanctuary ordinance conflict; Immigration enforcement access risk; State audit context</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>Board voted to cancel after concerns federal immigration agents could access village data contrary to sanctuary ordinance; shut off cameras.</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>https://www.oakpark.com/2025/12/02/new-reports-emerge-on-border-patrol-use-of-flock-cameras/</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>Verified local press</t>
         </is>
       </c>
+      <c r="N21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-021</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Eugene</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Unauthorized reactivation; Public pressure; Trust failure</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Terminated after a camera was reactivated without authorization; PD learned via community tip. Ended amid sustained local pressure.</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>https://www.klcc.org/breaking/2025-12-05/eugene-and-springfield-both-announce-end-of-flock-camera-usage</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>CAN-2025-022</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Springfield</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Public pressure; Cameras never turned on; Covered then removed</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>Same Dec. 2025 announcement wave as Eugene: Springfield said cameras had not been turned on and would be covered then removed after months of public pushback.</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>https://www.klcc.org/breaking/2025-12-05/eugene-and-springfield-both-announce-end-of-flock-camera-usage</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L23" s="3" t="inlineStr">
         <is>
           <t>https://www.npr.org/2026/02/17/nx-s1-5612825/flock-contracts-canceled-immigration-survillance-concerns</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M23" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-023</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Bend</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>4</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Security concerns; Federal compliance fears; Community opposition</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Council voted to remove four cameras citing security concerns and federal compliance fears.</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/news/flock-safety-rebellion-cities-canceling-federal-access-2026/</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
+      <c r="N24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>CAN-2025-024</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Talent</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Paused</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>2025-12-26</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>Immigration enforcement / sanctuary law fears; Community pressure</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>Unanimously paused cameras over concern data could be used for immigration enforcement contrary to Oregon sanctuary norms.</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/articles/surveillance/communities-winning-against-alpr-flock-safety-2025/</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="L25" s="3" t="inlineStr"/>
+      <c r="M25" s="3" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="N25" s="3" t="inlineStr">
         <is>
           <t>Pause may not equal permanent cancel.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-025</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Lynnwood</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Out-of-state agencies accessing network; Chief discovery after go-live</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>First Washington city reported to cancel an active Flock contract after chief discovered out-of-state agencies accessing the network.</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>https://mynorthwest.com/local/lynnwood-first-wa-city-cancel-flock-safety/4145920</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
+      <c r="N26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>CAN-2025-026</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Mountlake Terrace</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Pre-install cancel</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>Council vote before install; Community opposition climate</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>Unanimous council vote to end contract before cameras were installed.</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>https://www.heraldnet.com/news/mountlake-terrace-cancels-flock-safety-contract/</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-027</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Olympia</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>15</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>Public opposition; Pilot canceled; Cameras uninstalled</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Uninstalled ~15 cameras and canceled pilot program December 2025.</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>https://komonews.com/news/local/washington-cities-face-financial-questions-after-pausing-flock-camera-contracts</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
+      <c r="N28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>CAN-2025-028</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Redmond</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>Suspended</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>2025-11</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>Resident complaints; Contract reevaluation</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>Deactivated cameras November 2025 while reevaluating contract after resident complaints.</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>https://komonews.com/news/local/washington-cities-face-financial-questions-after-pausing-flock-camera-contracts</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L29" s="3" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M29" s="3" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="N29" s="3" t="inlineStr">
         <is>
           <t>May be pause rather than final cancel.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-029</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Windsor</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>16</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Public backlash; Resident campaign; Push for ALPR ban ordinance</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Town council voted to end contract; cameras turned off, removal planned. Resident organizer gathering petition signatures for ALPR ban ordinance.</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>https://www.nbcconnecticut.com/news/local/two-towns-end-contracts-with-automated-license-plate-reader-company-flock-safety/3755508/</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>Verified local TV</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>Physical removal scheduled into fall.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-030</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Killingworth</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Non-renewal</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>4</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>Security and privacy concerns; FOIA / records burden; Post-contract information about Flock</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>Not renewing four cameras on Route 81. First selectman said more information about Flock emerged after boards had already approved; FOIA handling concerns.</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>https://www.nbcconnecticut.com/news/local/two-towns-end-contracts-with-automated-license-plate-reader-company-flock-safety/3755508/</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="L31" s="3" t="inlineStr"/>
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>Verified local TV</t>
         </is>
       </c>
+      <c r="N31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-031</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Dayton</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>OH</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Suspended</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>2026-05</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>72</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Immigration-related search traffic vs city policy; Public demand for removal; Policy violations</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>Suspended fixed-site Flock program after review found immigration-related search activity against city policy. City covered ~72 cameras with bags; commissioners called for removal pending audit.</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>https://www.daytondailynews.com/local/city-covers-all-flock-cameras-amid-program-suspension/article_01aa7687-f68e-5443-b102-d98dd38ed9b6.html</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>https://www.businessinsider.com/cities-putting-trash-bags-over-flock-license-plate-readers-2026-6</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>Suspension + bags; final removal decision pending audit/commission.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-032</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Foothill-De Anza Community College District</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>2026-02-15</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>Discontinued program; Data sharing disabled; Privacy climate</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>Discontinued contract; covered lenses and disabled data sharing.</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="L33" s="3" t="inlineStr"/>
+      <c r="M33" s="3" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
+      <c r="N33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-033</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Hays County</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>2025-10</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Community opposition wave; Privacy / sharing concerns</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Contract terminated October 2025 amid Texas cancel wave following Austin-area organizing.</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/articles/surveillance/communities-winning-against-alpr-flock-safety-2025/</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>https://www.oakpark.com/2025/12/02/new-reports-emerge-on-border-patrol-use-of-flock-cameras/</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
+      <c r="N34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>CAN-2025-034</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>San Marcos</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Expired</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>Tied council vote; Community opposition</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>Contract lapsed after reported 3-3 vote dynamics; listed among Texas communities ending Flock use.</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K35" s="3" t="inlineStr">
         <is>
           <t>https://stateofsurveillance.org/articles/surveillance/communities-winning-against-alpr-flock-safety-2025/</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="L35" s="3" t="inlineStr"/>
+      <c r="M35" s="3" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
+      <c r="N35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-035</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Hillsborough</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>Privacy / federal access climate; Community opposition</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>Frequently listed among early cancelers in national roundups alongside Oak Park / Evanston wave.</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>https://www.oakpark.com/2025/12/02/new-reports-emerge-on-border-patrol-use-of-flock-cameras/</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>https://www.businessinsider.com/flock-safety-cameras-police-departments-lapd-2026-7</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
+      <c r="N36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>CAN-2025-036</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Natick</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>Data sharing / oversight concerns; Regional MA cancel wave</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J37" s="3" t="inlineStr">
         <is>
           <t>Boston.com reports Natick ended Flock contract alongside Cambridge and Watertown before Framingham non-renewal.</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K37" s="3" t="inlineStr">
         <is>
           <t>https://www.boston.com/news/local-news/2026/06/25/framingham-police-will-not-renew-flock-safety-contract-after-months-of-resident-opposition/</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="L37" s="3" t="inlineStr"/>
+      <c r="M37" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-037</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Watertown</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>Data sharing / oversight concerns; Regional MA cancel wave</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Boston.com reports Watertown ended Flock contract in the Massachusetts wave preceding Framingham.</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>https://www.boston.com/news/local-news/2026/06/25/framingham-police-will-not-renew-flock-safety-contract-after-months-of-resident-opposition/</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>CAN-2025-038</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Saranac Lake (Village)</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>Privacy concerns; Community opposition</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J39" s="3" t="inlineStr">
         <is>
           <t>Cited by WRVO among municipalities that voted to stop or pause Flock relationships before Ithaca.</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K39" s="3" t="inlineStr">
         <is>
           <t>https://www.wrvo.org/2026-03-05/ithaca-common-council-votes-to-end-contract-with-flock-safety</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="L39" s="3" t="inlineStr"/>
+      <c r="M39" s="3" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
+      <c r="N39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>CAN-2025-039</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Sedona</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>AZ</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>Privacy / immigration access climate</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>Listed with Flagstaff-era Arizona exits in Oak Park / regional reporting.</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>https://www.oakpark.com/2025/12/02/new-reports-emerge-on-border-patrol-use-of-flock-cameras/</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
+      <c r="N40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-040</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>El Cerrito</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>Bay Area cancel wave; Sanctuary / privacy climate</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J41" s="3" t="inlineStr">
         <is>
           <t>SF Standard reports El Cerrito ended its contract in the Bay Area wave (Mountain View, Santa Cruz, Campbell, Los Altos Hills, Santa Clara County).</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="3" t="inlineStr">
         <is>
           <t>https://sfstandard.com/2026/05/11/flock-safety-berkeley-sanctuary-city-contract/</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="L41" s="3" t="inlineStr"/>
+      <c r="M41" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>CAN-2026-041</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Santa Clara County</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>Bay Area cancel wave; Privacy / data-sharing scrutiny</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>SF Standard lists Santa Clara County among Bay Area jurisdictions that left Flock.</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>https://sfstandard.com/2026/05/11/flock-safety-berkeley-sanctuary-city-contract/</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>https://www.businessinsider.com/flock-safety-cameras-police-departments-lapd-2026-7</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
+      <c r="N42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>CAN-2026-042</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Campbell / Los Altos Hills (Bay Area cluster)</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>Terminated</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr"/>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
         <is>
           <t>Bay Area cancel wave; Public / sanctuary climate</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J43" s="3" t="inlineStr">
         <is>
           <t>SF Standard names Campbell and Los Altos Hills among more than a dozen California jurisdictions terminating Flock contracts.</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="3" t="inlineStr">
         <is>
           <t>https://sfstandard.com/2026/05/11/flock-safety-berkeley-sanctuary-city-contract/</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="L43" s="3" t="inlineStr"/>
+      <c r="M43" s="3" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
+      <c r="N43" s="3" t="inlineStr">
         <is>
           <t>Cluster row; split to separate Case_IDs when local minutes located.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>CAN-2026-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Fort Collins</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Terminated</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Public backlash; Pause on new ALPR bids until citywide surveillance policy; Physical removal</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>City Council voted 6–1 on June 16, 2026 to immediately cancel Flock, stop data collection, remove cameras, and delay new ALPR bids until a citywide surveillance policy exists. Staff confirmed all 15 city Flock cameras removed by early July 2026.</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.coloradoan.com/story/news/local/2026/06/16/fort-collins-to-immediately-end-contract-with-flock-safety/90584281007/</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.coloradoan.com/story/news/local/2026/07/23/fort-collins-police-services-flock-safety-cameras-have-been-removed/91021962007/</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>Private Flock cameras elsewhere in area not covered by city vote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>CAN-2026-044</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Harrisonburg</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Terminated</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Public backlash; Fixed-ALPR policy requiring council approval; Organized opposition (Deflock Harrisonburg)</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Harrisonburg City Council voted 4–0 on July 29, 2026 to end the Flock contract and adopt a policy generally prohibiting mounted ALPRs without express council approval. About 31 Falcon cameras; systems to go dark ~July 31 with removal work order.</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.29news.com/2026/07/29/harrisonburg-city-council-votes-end-contract-with-flock-safety/</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.dnronline.com/news/public_safety/harrisonburg-city-council-votes-to-cancel-flock-camera-contract/article_e96103ea-5a30-5d31-9d9c-3198e8ae5c9e.html</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="inlineStr">
+        <is>
+          <t>Broader ban on all future mass-surveillance vendors not passed in same vote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>CAN-2026-045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Elkton</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Terminated</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Regional Shenandoah Valley cancel wave; Public backlash</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Elkton ended its Flock contract the week before Harrisonburg’s July 29, 2026 cancel, per regional coverage of the Shenandoah Valley exit wave (alongside earlier Staunton / Charlottesville exits).</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dnronline.com/news/public_safety/harrisonburg-city-council-votes-to-cancel-flock-camera-contract/article_e96103ea-5a30-5d31-9d9c-3198e8ae5c9e.html</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.29news.com/2026/07/29/harrisonburg-city-council-votes-end-contract-with-flock-safety/</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>Camera count and exact council vote date not detailed in Harrisonburg-focused coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>CAN-2026-046</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Non-renewal</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr"/>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Data ownership / local-control concerns; Seeking replacement vendor</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>Salem Mayor Dominick Pangallo and Police Chief Lucas Miller said the city would not renew Flock and would remove installed ALPRs over insufficient data protections, while seeking systems that better retain local control — a cancel-then-replace risk pattern.</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.boston.com/news/local-news/2026/07/26/salem-joins-list-of-mass-communities-to-reject-surveillance-company-over-data-concerns/</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wcvb.com/article/flock-camera-contract-ending-salem-ma-july-24/73258537</t>
+        </is>
+      </c>
+      <c r="M47" s="3" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N47" s="3" t="inlineStr">
+        <is>
+          <t>City indicated intent to replace with another ALPR vendor retaining local data control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>CAN-2026-047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Monroe County</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Terminated</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Privacy / mass-surveillance concerns; Outside and federal access risk; Physical removal emphasis</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Monroe County Commissioners voted to cancel the Flock contract (~6 cameras), citing privacy and mass-surveillance concerns and risk that plate/location data could be accessed by outside or federal agencies. Coverage notes Bloomington also ending its Flock contract; officials emphasized cameras must come down, not only contracts ending. CBS4 Indy / WIBC / WBIW July 28, 2026.</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>https://cbs4indy.com/news/monroe-county-ditches-flock-cameras-citing-privacy-concerns/</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>https://wibc.com/893233/monroe-county-ditches-flock-cameras-over-privacy-concerns/</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>YouTube: https://www.youtube.com/watch?v=eguU9gQfZ54 (CBS4 Indy). Bloomington city exit tracked separately (CAN-2026-017).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>CAN-2026-048</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Stoughton</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Terminated</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Public backlash; Privacy concerns; Early buyout of two-year contract</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Stoughton City Council unanimously voted July 28, 2026 to terminate Flock after months of resident opposition. Five cameras (four ALPR + one live feed); ~$12,500 remaining buyout on a two-year/$25,000 contract; removal and data deletion directed; commitment not to swap to similar tech without 30 days’ notice and public input. Seventh Dane County entity ending Flock per local reporting.</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wmtv15news.com/2026/07/29/stoughton-city-council-unanimously-votes-terminate-agreement-with-flock-safety/</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.channel3000.com/news/stoughton-council-members-vote-to-terminate-flock-contract/article_cd05b0a6-881a-48ef-b0d2-bddb24d2a343.html</t>
+        </is>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N49" s="3" t="inlineStr">
+        <is>
+          <t>YouTube: https://www.youtube.com/watch?v=4NtGB6BMvFU (WKOW 27). WKOW video page: https://www.wkow.com/video/stoughton-votes-to-remove-flock-cameras/video_5cb9e98e-a618-5f0b-bff7-71342db8f8c6.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>CAN-2026-049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>South Kingstown</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>RI</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Terminated</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Public backlash; Privacy concerns; ACLU of RI advocacy letter; Misuse/federal-access fears</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>South Kingstown Town Council voted unanimously (5–0) on July 27, 2026 to terminate Flock and remove cameras ASAP after hundreds of resident emails and an ACLU of Rhode Island letter. Contract ~$30,300/year; ~6–7 cameras active since Feb 2026. Seeking partial refund. State Police Flock on state roads may remain nearby.</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wpri.com/news/local-news/south-county/south-kingstown-to-stop-using-automated-license-plate-readers/</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>https://turnto10.com/news/local/south-kingstown-ends-partnership-with-flock-cameras-july-28-2026</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>YouTube WPRI https://www.youtube.com/watch?v=5a4l65Jen3E and WJAR https://www.youtube.com/watch?v=9RRqBtry1CU cover the same South Kingstown cancel. ACLU RI: https://www.riaclu.org/news/south-kingstown-cancels-flock-safety-contract-after-community-advocacy-aclu-letter/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Leon grant reject, ALPR Week of Action, and Coffee/Niceville misuse panels.
Sync cancel dossier to 61 records and refresh Mooresville/Rozar/Hall misuse rows with regenerated Excel/PDF tallies.
</commit_message>
<xml_diff>
--- a/docs/Flock_Municipal_Cancellations_Database.xlsx
+++ b/docs/Flock_Municipal_Cancellations_Database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N61"/>
+  <dimension ref="A1:N62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4347,6 +4347,73 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CAN-2026-061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Leon County</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Pre-install cancel</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Public backlash; Privacy / surveillance concerns; Regional grant reject</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Leon County Commission on July 14, 2026 unanimously stripped about $440,000 in regional public-safety grant funding that would have expanded Flock ALPRs in neighboring Wakulla, Jefferson, Liberty, and Taylor counties (pass-through via Leon County Sheriff’s Office). Commissioners approved other grant items, directed a September workshop on county authority to regulate or ban ALPRs locally, after packed public comment opposing surveillance expansion.</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>https://www.tallahassee.com/story/news/local/2026/07/16/leon-county-rejects-grants-for-flock-license-plate-readers/90930124007/</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>https://news.wfsu.org/wfsu-local-news/2026-07-14/leon-commissioners-pass-data-center-moratorium-block-flock-camera-grant-funding</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Rejects regional expansion grant funding, not removal of existing Leon County cameras; September 2026 authority/workshop follow-up pending.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync cancel/misuse/wrongful dossiers with site panels and refresh tallies.
Catch up Syracuse, Charlottesville, and Grand Chute cancel rows that landed on HTML first, regenerate exports, and realign Case_ID cites and as-of counts.
</commit_message>
<xml_diff>
--- a/docs/Flock_Municipal_Cancellations_Database.xlsx
+++ b/docs/Flock_Municipal_Cancellations_Database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1723,35 +1723,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAN-2026-001</t>
+          <t>CAN-2025-040</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Oshkosh</t>
+          <t>Charlottesville</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>WI</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Rescinded</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>26</v>
+          <t>2025-12</t>
+        </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1761,44 +1758,40 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Vendor misrepresentation (heat maps); Police chief trust failure; Public backlash</t>
+          <t>Public backlash; Regional Virginia cancel wave</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Council approved a one-year renewal amid vocal public opposition, then unanimously rescinded within ~24 hours after Police Chief Dean Smith said Flock misrepresented heat-map tracking capability at the council meeting. Cameras powered off and bagged.</t>
+          <t>Charlottesville terminated its Flock contract in December 2025. Later Shenandoah / central Virginia coverage (including Harrisonburg’s July 2026 cancel) cites Charlottesville alongside Staunton as earlier exits in the same regional wave.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.postcrescent.com/story/news/local/oshkosh/2026/04/22/oshkosh-rescinds-flock-safety-contract-after-police-chief-raises-concerns/89745485007/</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>https://www.wbay.com/2026/04/23/oshkosh-council-rescinds-flock-camera-contract-after-false-statements/</t>
-        </is>
-      </c>
+          <t>https://www.dnronline.com/news/public_safety/harrisonburg-city-council-votes-to-cancel-flock-camera-contract/article_e96103ea-5a30-5d31-9d9c-3198e8ae5c9e.html</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Verified major press</t>
+          <t>Verified secondary press</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Hardware bagged while removal coordinated.</t>
+          <t>Date and exit confirmed in later regional reporting tied to Harrisonburg coverage; add a Charlottesville-primary URL when one is catalogued.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAN-2026-002</t>
+          <t>CAN-2026-001</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Verona</t>
+          <t>Oshkosh</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1808,13 +1801,16 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Non-renewal</t>
+          <t>Rescinded</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2025-12</t>
-        </is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>26</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1828,17 +1824,22 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Public backlash; Loss of trust in vendor (not PD); Data-sharing / federal access fears</t>
+          <t>Vendor misrepresentation (heat maps); Police chief trust failure; Public backlash</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Common Council voted not to renew; contract lapsed December. Officials and residents framed the decision as lack of public trust in Flock Safety. Cameras remained up for months; city covered them pending physical removal.</t>
+          <t>Council approved a one-year renewal amid vocal public opposition, then unanimously rescinded within ~24 hours after Police Chief Dean Smith said Flock misrepresented heat-map tracking capability at the council meeting. Cameras powered off and bagged.</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://wisconsinexaminer.com/2026/02/02/verona-expected-to-begin-work-to-removing-flock-cameras/</t>
+          <t>https://www.postcrescent.com/story/news/local/oshkosh/2026/04/22/oshkosh-rescinds-flock-safety-contract-after-police-chief-raises-concerns/89745485007/</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.wbay.com/2026/04/23/oshkosh-council-rescinds-flock-camera-contract-after-false-statements/</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1848,24 +1849,24 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Physical removal lagged contract end; interim lens covers.</t>
+          <t>Hardware bagged while removal coordinated.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAN-2026-004</t>
+          <t>CAN-2026-002</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Framingham</t>
+          <t>Verona</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>WI</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1875,12 +1876,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1890,17 +1891,17 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Public backlash; Resident advocacy; Data sharing / oversight concerns</t>
+          <t>Public backlash; Loss of trust in vendor (not PD); Data-sharing / federal access fears</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Police will not renew after months of resident opposition. System access shut off at contract end; Flock to remove cameras. Follows Cambridge, Watertown, and Natick exits in Massachusetts.</t>
+          <t>Common Council voted not to renew; contract lapsed December. Officials and residents framed the decision as lack of public trust in Flock Safety. Cameras remained up for months; city covered them pending physical removal.</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://www.boston.com/news/local-news/2026/06/25/framingham-police-will-not-renew-flock-safety-contract-after-months-of-resident-opposition/</t>
+          <t>https://wisconsinexaminer.com/2026/02/02/verona-expected-to-begin-work-to-removing-flock-cameras/</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -1910,24 +1911,24 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Advocates seeking assurance city will not replace with similar system.</t>
+          <t>Physical removal lagged contract end; interim lens covers.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAN-2026-006</t>
+          <t>CAN-2026-004</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Westland</t>
+          <t>Framingham</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1937,11 +1938,8 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>10</v>
+          <t>2026-06-30</t>
+        </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1955,55 +1953,58 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Public backlash; Privacy / constitutional concerns; Outside agency / ICE access fears; Split council</t>
+          <t>Public backlash; Resident advocacy; Data sharing / oversight concerns</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Police chief did not bring renewal to council after finding council deeply split. Council president cited privacy, corporate sharing, ICE access fears, and credited residents and advocacy groups for raising concerns.</t>
+          <t>Police will not renew after months of resident opposition. System access shut off at contract end; Flock to remove cameras. Follows Cambridge, Watertown, and Natick exits in Massachusetts.</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://www.clickondetroit.com/news/local/2026/07/10/westland-to-remove-flock-safety-license-plate-cameras-after-privacy-concerns/</t>
+          <t>https://www.boston.com/news/local-news/2026/06/25/framingham-police-will-not-renew-flock-safety-contract-after-months-of-resident-opposition/</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Verified local TV</t>
+          <t>Verified major press</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Removal at contract expiration end of month.</t>
+          <t>Advocates seeking assurance city will not replace with similar system.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAN-2026-007</t>
+          <t>CAN-2026-006</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ithaca</t>
+          <t>Westland</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Terminated</t>
+          <t>Non-renewal</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-03</t>
-        </is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>10</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2017,39 +2018,44 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Public backlash; Sanctuary-city conflict; Third-party disclosure language; Outside agency access concerns</t>
+          <t>Public backlash; Privacy / constitutional concerns; Outside agency / ICE access fears; Split council</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Common Council ended the contract after activist campaign and protests outside city hall. Resolution cited sanctuary policies and documented outside-agency access without explicit local authorization.</t>
+          <t>Police chief did not bring renewal to council after finding council deeply split. Council president cited privacy, corporate sharing, ICE access fears, and credited residents and advocacy groups for raising concerns.</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://www.wrvo.org/2026-03-05/ithaca-common-council-votes-to-end-contract-with-flock-safety</t>
+          <t>https://www.clickondetroit.com/news/local/2026/07/10/westland-to-remove-flock-safety-license-plate-cameras-after-privacy-concerns/</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Verified major press</t>
+          <t>Verified local TV</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Removal at contract expiration end of month.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAN-2026-008</t>
+          <t>CAN-2026-007</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Santa Cruz</t>
+          <t>Ithaca</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2059,7 +2065,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2074,22 +2080,17 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Out-of-state access; Immigration / sanctuary urgency; Public / grassroots pressure (Get the Flock Out)</t>
+          <t>Public backlash; Sanctuary-city conflict; Third-party disclosure language; Outside agency access concerns</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Council voted 6-1 to terminate after out-of-state agencies accessed city data. Widely reported as first California city to end a Flock contract; grassroots organizing credited alongside immigration-enforcement urgency.</t>
+          <t>Common Council ended the contract after activist campaign and protests outside city hall. Resolution cited sanctuary policies and documented outside-agency access without explicit local authorization.</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://www.kqed.org/news/12069705/santa-cruz-the-first-in-california-to-terminate-its-contract-with-flock-safety</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>https://www.npr.org/2026/02/17/nx-s1-5612825/flock-contracts-canceled-immigration-survillance-concerns</t>
+          <t>https://www.wrvo.org/2026-03-05/ithaca-common-council-votes-to-end-contract-with-flock-safety</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2101,17 +2102,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAN-2026-009</t>
+          <t>CAN-2026-008</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>South Portland</t>
+          <t>Santa Cruz</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2121,11 +2122,8 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>7</v>
+          <t>2026-01</t>
+        </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -2139,58 +2137,58 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Public backlash; Privacy / constitutional concerns</t>
+          <t>Out-of-state access; Immigration / sanctuary urgency; Public / grassroots pressure (Get the Flock Out)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Council workshop directed end of Flock use after strong community backlash. All seven cameras removed by June 22, 2026; no active South Portland Flock account.</t>
+          <t>Council voted 6-1 to terminate after out-of-state agencies accessed city data. Widely reported as first California city to end a Flock contract; grassroots organizing credited alongside immigration-enforcement urgency.</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://www.southportland.gov/m/NewsFlash/home/detail/550</t>
+          <t>https://www.kqed.org/news/12069705/santa-cruz-the-first-in-california-to-terminate-its-contract-with-flock-safety</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.pressherald.com/2026/07/01/south-portlands-flock-cameras-have-been-removed/</t>
+          <t>https://www.npr.org/2026/02/17/nx-s1-5612825/flock-contracts-canceled-immigration-survillance-concerns</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Verified local/primary</t>
+          <t>Verified major press</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAN-2026-010</t>
+          <t>CAN-2026-009</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>South Portland</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Expired</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>110</v>
+        <v>7</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -2204,58 +2202,58 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Public backlash; Privacy concerns; Federal immigration data-sharing revelations</t>
+          <t>Public backlash; Privacy / constitutional concerns</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Largest reported single municipal removal by camera count: 110 intersection cameras decommissioned and removed when contract expired. City approved Axon replacement (~50 cams) with stricter controls.</t>
+          <t>Council workshop directed end of Flock use after strong community backlash. All seven cameras removed by June 22, 2026; no active South Portland Flock account.</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://www.9news.com/article/news/local/denver-removes-flock-license-plate-reader-cameras/73-eaf91d0a-3b90-45f5-8338-dbb9f79a8712</t>
+          <t>https://www.southportland.gov/m/NewsFlash/home/detail/550</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://www.pressherald.com/2026/07/01/south-portlands-flock-cameras-have-been-removed/</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Verified local TV</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Private/HOA Flock cameras remain; some pre-Flock city LPR gear unaffected.</t>
+          <t>Verified local/primary</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAN-2026-013</t>
+          <t>CAN-2026-010</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Mountain View</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Suspended</t>
+          <t>Expired</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>30</v>
+        <v>110</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -2264,44 +2262,44 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Unauthorized federal access (ATF; Air Force; GSA IG); Audit findings</t>
+          <t>Public backlash; Privacy concerns; Federal immigration data-sharing revelations</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Disabled all ~30 cameras after audit showed federal agencies had accessed local data without authorization.</t>
+          <t>Largest reported single municipal removal by camera count: 110 intersection cameras decommissioned and removed when contract expired. City approved Axon replacement (~50 cams) with stricter controls.</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://localnewsmatters.org/2026/03/03/mountain-view-terminates-license-plate-reader-contract-with-flock-safety/</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
+          <t>https://www.9news.com/article/news/local/denver-removes-flock-license-plate-reader-cameras/73-eaf91d0a-3b90-45f5-8338-dbb9f79a8712</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Verified major press</t>
+          <t>Verified local TV</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Private/HOA Flock cameras remain; some pre-Flock city LPR gear unaffected.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAN-2026-014</t>
+          <t>CAN-2026-013</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Oxnard</t>
+          <t>Mountain View</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2316,11 +2314,11 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2334,44 +2332,39 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Vendor-enabled National Lookup vs California law; Out-of-state / federal queries; Public trust</t>
+          <t>Unauthorized federal access (ATF; Air Force; GSA IG); Audit findings</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>OPD suspended 19 fixed Flock cameras after audit found nationwide query capability allowed out-of-state/federal agencies to include Oxnard data despite California-only settings.</t>
+          <t>Disabled all ~30 cameras after audit showed federal agencies had accessed local data without authorization.</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://www.oxnard.gov/pd-news/news-release-oxnard-police-department-suspends-use-of-flock-safety-automated-license-plate-readers-02-27-26</t>
+          <t>https://localnewsmatters.org/2026/03/03/mountain-view-terminates-license-plate-reader-contract-with-flock-safety/</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.edhat.com/ventura/news/oxnard-police-suspend-flock-license-plate-readers-ventura-agencies-tighten-controls-after-out-of-state-access/</t>
+          <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Verified local/primary</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Suspension pending confidence in safeguards; not necessarily permanent cancel.</t>
+          <t>Verified major press</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAN-2026-015</t>
+          <t>CAN-2026-014</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>South Pasadena</t>
+          <t>Oxnard</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2381,16 +2374,16 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Terminated</t>
+          <t>Suspended</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2404,34 +2397,44 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Privacy concerns; Illegal sharing with federal immigration agents (regional reports)</t>
+          <t>Vendor-enabled National Lookup vs California law; Out-of-state / federal queries; Public trust</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Council canceled contract for ~14 cameras after reports Southern California agencies shared Flock data with federal immigration agents.</t>
+          <t>OPD suspended 19 fixed Flock cameras after audit found nationwide query capability allowed out-of-state/federal agencies to include Oxnard data despite California-only settings.</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://laist.com/news/politics/south-pasadena-cancels-contract-with-flock-safety-citing-privacy-concerns</t>
+          <t>https://www.oxnard.gov/pd-news/news-release-oxnard-police-department-suspends-use-of-flock-safety-automated-license-plate-readers-02-27-26</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://www.edhat.com/ventura/news/oxnard-police-suspend-flock-license-plate-readers-ventura-agencies-tighten-controls-after-out-of-state-access/</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Verified major press</t>
+          <t>Verified local/primary</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Suspension pending confidence in safeguards; not necessarily permanent cancel.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAN-2026-016</t>
+          <t>CAN-2026-015</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Los Angeles Police Department</t>
+          <t>South Pasadena</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2441,16 +2444,16 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Expired</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>138</v>
+        <v>14</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -2464,49 +2467,39 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Privacy / civil liberties; Data ownership uncertainty; Federal access concerns</t>
+          <t>Privacy concerns; Illegal sharing with federal immigration agents (regional reports)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>LAPD let three-year agreement expire (~138 pole cameras since 2023). Audit/reporting cited federal access and immigration-enforcement risk. Some outlets note possible renegotiation with stricter terms.</t>
+          <t>Council canceled contract for ~14 cameras after reports Southern California agencies shared Flock data with federal immigration agents.</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://www.businessinsider.com/flock-safety-cameras-police-departments-lapd-2026-7</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>https://www.cnet.com/news/privacy/los-angeles-lapd-flock-safety-surveillance-cameras-privacy/</t>
+          <t>https://laist.com/news/politics/south-pasadena-cancels-contract-with-flock-safety-citing-privacy-concerns</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
           <t>Verified major press</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>May renegotiate; not necessarily a permanent ban.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAN-2026-017</t>
+          <t>CAN-2026-016</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Bloomington</t>
+          <t>Los Angeles Police Department</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2516,8 +2509,11 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
-        </is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>138</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -2531,53 +2527,60 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Months-long evaluation; Oversight / legal considerations; Council oversight resolution context</t>
+          <t>Privacy / civil liberties; Data ownership uncertainty; Federal access concerns</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Mayor announced contract expired and city would not renew after evaluation with PD, legal, Flock, and community partners. Sharing narrowed during wind-down.</t>
+          <t>LAPD let three-year agreement expire (~138 pole cameras since 2023). Audit/reporting cited federal access and immigration-enforcement risk. Some outlets note possible renegotiation with stricter terms.</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://bloomington.in.gov/news/2026/04/15/6521</t>
+          <t>https://www.businessinsider.com/flock-safety-cameras-police-departments-lapd-2026-7</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.cnet.com/news/privacy/los-angeles-lapd-flock-safety-surveillance-cameras-privacy/</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Verified local/primary</t>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>May renegotiate; not necessarily a permanent ban.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAN-2026-018</t>
+          <t>CAN-2026-017</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Edmonds</t>
+          <t>Bloomington</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Terminated</t>
+          <t>Expired</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>19</v>
+          <t>2026-03-05</t>
+        </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2591,39 +2594,39 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>New state ALPR law compliance; Retention / audit / disclosure liability; Staffing burden</t>
+          <t>Months-long evaluation; Oversight / legal considerations; Council oversight resolution context</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Council unanimously authorized termination after procedural correction. Chief cited new state guardrails creating liability and records burdens.</t>
+          <t>Mayor announced contract expired and city would not renew after evaluation with PD, legal, Flock, and community partners. Sharing narrowed during wind-down.</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>https://www.heraldnet.com/2026/06/10/following-procedural-error-edmonds-unanimously-cancels-flock-contract/</t>
+          <t>https://bloomington.in.gov/news/2026/04/15/6521</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Verified major press</t>
+          <t>Verified local/primary</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAN-2026-023</t>
+          <t>CAN-2026-018</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bend</t>
+          <t>Edmonds</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OR</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2633,11 +2636,11 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2646,44 +2649,44 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Security concerns; Federal compliance fears; Community opposition</t>
+          <t>New state ALPR law compliance; Retention / audit / disclosure liability; Staffing burden</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Council voted to remove four cameras citing security concerns and federal compliance fears.</t>
+          <t>Council unanimously authorized termination after procedural correction. Chief cited new state guardrails creating liability and records burdens.</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>https://stateofsurveillance.org/news/flock-safety-rebellion-cities-canceling-federal-access-2026/</t>
+          <t>https://www.heraldnet.com/2026/06/10/following-procedural-error-edmonds-unanimously-cancels-flock-contract/</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Aggregator-aligned (confirm)</t>
+          <t>Verified major press</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAN-2026-029</t>
+          <t>CAN-2026-023</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Windsor</t>
+          <t>Bend</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2693,11 +2696,11 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2711,39 +2714,34 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Public backlash; Resident campaign; Push for ALPR ban ordinance</t>
+          <t>Security concerns; Federal compliance fears; Community opposition</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Town council voted to end contract; cameras turned off, removal planned. Resident organizer gathering petition signatures for ALPR ban ordinance.</t>
+          <t>Council voted to remove four cameras citing security concerns and federal compliance fears.</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>https://www.nbcconnecticut.com/news/local/two-towns-end-contracts-with-automated-license-plate-reader-company-flock-safety/3755508/</t>
+          <t>https://stateofsurveillance.org/news/flock-safety-rebellion-cities-canceling-federal-access-2026/</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Verified local TV</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Physical removal scheduled into fall.</t>
+          <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAN-2026-030</t>
+          <t>CAN-2026-029</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Killingworth</t>
+          <t>Windsor</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2753,7 +2751,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Non-renewal</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2762,7 +2760,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2771,17 +2769,17 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Security and privacy concerns; FOIA / records burden; Post-contract information about Flock</t>
+          <t>Public backlash; Resident campaign; Push for ALPR ban ordinance</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Not renewing four cameras on Route 81. First selectman said more information about Flock emerged after boards had already approved; FOIA handling concerns.</t>
+          <t>Town council voted to end contract; cameras turned off, removal planned. Resident organizer gathering petition signatures for ALPR ban ordinance.</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2792,37 +2790,42 @@
       <c r="M38" t="inlineStr">
         <is>
           <t>Verified local TV</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Physical removal scheduled into fall.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAN-2026-031</t>
+          <t>CAN-2026-030</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dayton</t>
+          <t>Killingworth</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Suspended</t>
+          <t>Non-renewal</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2831,65 +2834,58 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Immigration-related search traffic vs city policy; Public demand for removal; Policy violations</t>
+          <t>Security and privacy concerns; FOIA / records burden; Post-contract information about Flock</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Suspended fixed-site Flock program after review found immigration-related search activity against city policy. City covered ~72 cameras with bags; commissioners called for removal pending audit.</t>
+          <t>Not renewing four cameras on Route 81. First selectman said more information about Flock emerged after boards had already approved; FOIA handling concerns.</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>https://www.daytondailynews.com/local/city-covers-all-flock-cameras-amid-program-suspension/article_01aa7687-f68e-5443-b102-d98dd38ed9b6.html</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>https://www.businessinsider.com/cities-putting-trash-bags-over-flock-license-plate-readers-2026-6</t>
+          <t>https://www.nbcconnecticut.com/news/local/two-towns-end-contracts-with-automated-license-plate-reader-company-flock-safety/3755508/</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Verified major press</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Suspension + bags; final removal decision pending audit/commission.</t>
+          <t>Verified local TV</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAN-2026-032</t>
+          <t>CAN-2026-031</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Foothill-De Anza Community College District</t>
+          <t>Dayton</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Terminated</t>
+          <t>Suspended</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
-        </is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>72</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2898,39 +2894,49 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Discontinued program; Data sharing disabled; Privacy climate</t>
+          <t>Immigration-related search traffic vs city policy; Public demand for removal; Policy violations</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Discontinued contract; covered lenses and disabled data sharing.</t>
+          <t>Suspended fixed-site Flock program after review found immigration-related search activity against city policy. City covered ~72 cameras with bags; commissioners called for removal pending audit.</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
+          <t>https://www.daytondailynews.com/local/city-covers-all-flock-cameras-amid-program-suspension/article_01aa7687-f68e-5443-b102-d98dd38ed9b6.html</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>https://www.businessinsider.com/cities-putting-trash-bags-over-flock-license-plate-readers-2026-6</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Aggregator-aligned (confirm)</t>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Suspension + bags; final removal decision pending audit/commission.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAN-2026-040</t>
+          <t>CAN-2026-032</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>El Cerrito</t>
+          <t>Foothill-De Anza Community College District</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2945,7 +2951,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2955,49 +2961,39 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Bay Area cancel wave; Sanctuary / privacy climate</t>
+          <t>Discontinued program; Data sharing disabled; Privacy climate</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>SF Standard reports El Cerrito ended its contract in the Bay Area wave (Mountain View, Santa Cruz, Campbell, Los Altos Hills, Santa Clara County).</t>
+          <t>Discontinued contract; covered lenses and disabled data sharing.</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>https://sfstandard.com/2026/05/11/flock-safety-berkeley-sanctuary-city-contract/</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>https://www.kalw.org/bay-area-news/2026-07-31/el-cerrito-begins-removing-flock-cameras</t>
+          <t>https://stateofsurveillance.org/news/flock-safety-cancel-wave-30-cities-alpr-surveillance-contracts-2026/</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Verified major press</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>Contract expired June 6, 2026 after May non-renewal. KALW reported July 31, 2026 that police began physically removing cameras; Flock told the city removal would run through about August 18. Residents had flagged units still flickering after supposed offline date.</t>
+          <t>Aggregator-aligned (confirm)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAN-2026-041</t>
+          <t>CAN-2026-040</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Santa Clara County</t>
+          <t>El Cerrito</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3007,59 +3003,64 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Terminated</t>
+          <t>Non-renewal</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Bay Area cancel wave; Privacy / data-sharing scrutiny</t>
+          <t>Unauthorized federal access; Public backlash; Sanctuary / privacy climate</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>SF Standard lists Santa Clara County among Bay Area jurisdictions that left Flock.</t>
+          <t>El Cerrito council voted in May 2026 not to renew after federal agencies accessed data from about 40 cameras without local police knowledge. The contract expired June 6; cameras were supposed to be offline, but residents flagged a unit still flickering. KALW reported July 31, 2026 that police began physically removing cameras; Flock told the city removal would run through about August 18.</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>https://sfstandard.com/2026/05/11/flock-safety-berkeley-sanctuary-city-contract/</t>
+          <t>https://ccpulse.org/2026/05/07/el-cerrito-becomes-first-in-county-to-drop-flock-after-unauthorized-searches/</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.businessinsider.com/flock-safety-cameras-police-departments-lapd-2026-7</t>
+          <t>https://www.kalw.org/bay-area-news/2026-07-31/el-cerrito-begins-removing-flock-cameras</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
           <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Contract expired June 6, 2026 after May non-renewal. KALW reported July 31, 2026 that police began physically removing cameras; Flock told the city removal would run through about August 18. Residents had flagged units still flickering after supposed offline date.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAN-2026-042</t>
+          <t>CAN-2026-041</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Campbell / Los Altos Hills (Bay Area cluster)</t>
+          <t>Santa Clara County</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3084,17 +3085,17 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Bay Area cancel wave; Public / sanctuary climate</t>
+          <t>Bay Area cancel wave; Privacy / data-sharing scrutiny</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>SF Standard names Campbell and Los Altos Hills among more than a dozen California jurisdictions terminating Flock contracts.</t>
+          <t>SF Standard lists Santa Clara County among Bay Area jurisdictions that left Flock.</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3102,31 +3103,31 @@
           <t>https://sfstandard.com/2026/05/11/flock-safety-berkeley-sanctuary-city-contract/</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>https://www.businessinsider.com/flock-safety-cameras-police-departments-lapd-2026-7</t>
+        </is>
+      </c>
       <c r="M43" t="inlineStr">
         <is>
           <t>Verified major press</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Cluster row; split to separate Case_IDs when local minutes located.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAN-2026-043</t>
+          <t>CAN-2026-042</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Fort Collins</t>
+          <t>Campbell / Los Altos Hills (Bay Area cluster)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3136,15 +3137,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="F44" t="n">
-        <v>15</v>
+          <t>2026</t>
+        </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3154,22 +3152,17 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Public backlash; Pause on new ALPR bids until citywide surveillance policy; Physical removal</t>
+          <t>Bay Area cancel wave; Public / sanctuary climate</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>City Council voted 6-1 on June 16, 2026 to immediately cancel Flock, stop data collection, remove cameras, and delay new ALPR bids until a citywide surveillance policy exists. Staff confirmed all 15 city Flock cameras removed by early July 2026.</t>
+          <t>SF Standard names Campbell and Los Altos Hills among more than a dozen California jurisdictions terminating Flock contracts.</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>https://www.coloradoan.com/story/news/local/2026/06/16/fort-collins-to-immediately-end-contract-with-flock-safety/90584281007/</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>https://www.coloradoan.com/story/news/local/2026/07/23/fort-collins-police-services-flock-safety-cameras-have-been-removed/91021962007/</t>
+          <t>https://sfstandard.com/2026/05/11/flock-safety-berkeley-sanctuary-city-contract/</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3179,24 +3172,24 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Private Flock cameras elsewhere in area not covered by city vote.</t>
+          <t>Cluster row; split to separate Case_IDs when local minutes located.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAN-2026-044</t>
+          <t>CAN-2026-043</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Harrisonburg</t>
+          <t>Fort Collins</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3206,11 +3199,11 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -3224,22 +3217,22 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Public backlash; Fixed-ALPR policy requiring council approval; Organized opposition (Deflock Harrisonburg)</t>
+          <t>Public backlash; Pause on new ALPR bids until citywide surveillance policy; Physical removal</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Harrisonburg City Council voted 4-0 on July 29, 2026 to end the Flock contract and adopt a policy generally prohibiting mounted ALPRs without express council approval. About 31 Falcon cameras; systems to go dark ~July 31 with removal work order.</t>
+          <t>City Council voted 6-1 on June 16, 2026 to immediately cancel Flock, stop data collection, remove cameras, and delay new ALPR bids until a citywide surveillance policy exists. Staff confirmed all 15 city Flock cameras removed by early July 2026.</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>https://www.29news.com/2026/07/29/harrisonburg-city-council-votes-end-contract-with-flock-safety/</t>
+          <t>https://www.coloradoan.com/story/news/local/2026/06/16/fort-collins-to-immediately-end-contract-with-flock-safety/90584281007/</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.dnronline.com/news/public_safety/harrisonburg-city-council-votes-to-cancel-flock-camera-contract/article_e96103ea-5a30-5d31-9d9c-3198e8ae5c9e.html</t>
+          <t>https://www.coloradoan.com/story/news/local/2026/07/23/fort-collins-police-services-flock-safety-cameras-have-been-removed/91021962007/</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3249,19 +3242,19 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Broader ban on all future mass-surveillance vendors not passed in same vote.</t>
+          <t>Private Flock cameras elsewhere in area not covered by city vote.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAN-2026-045</t>
+          <t>CAN-2026-044</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Elkton</t>
+          <t>Harrisonburg</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3276,12 +3269,15 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>31</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3291,24 +3287,24 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Regional Shenandoah Valley cancel wave; Public backlash</t>
+          <t>Public backlash; Fixed-ALPR policy requiring council approval; Organized opposition (Deflock Harrisonburg)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Elkton ended its Flock contract the week before Harrisonburg’s July 29, 2026 cancel, per regional coverage of the Shenandoah Valley exit wave (alongside earlier Staunton / Charlottesville exits).</t>
+          <t>Harrisonburg City Council voted 4-0 on July 29, 2026 to end the Flock contract and adopt a policy generally prohibiting mounted ALPRs without express council approval. About 31 Falcon cameras; systems to go dark ~July 31 with removal work order.</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
+          <t>https://www.29news.com/2026/07/29/harrisonburg-city-council-votes-end-contract-with-flock-safety/</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
           <t>https://www.dnronline.com/news/public_safety/harrisonburg-city-council-votes-to-cancel-flock-camera-contract/article_e96103ea-5a30-5d31-9d9c-3198e8ae5c9e.html</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>https://www.29news.com/2026/07/29/harrisonburg-city-council-votes-end-contract-with-flock-safety/</t>
-        </is>
-      </c>
       <c r="M46" t="inlineStr">
         <is>
           <t>Verified major press</t>
@@ -3316,29 +3312,29 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Camera count and exact council vote date not detailed in Harrisonburg-focused coverage.</t>
+          <t>Broader ban on all future mass-surveillance vendors not passed in same vote.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAN-2026-046</t>
+          <t>CAN-2026-045</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Salem</t>
+          <t>Elkton</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Non-renewal</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3348,7 +3344,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3358,22 +3354,22 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Data ownership / local-control concerns; Seeking replacement vendor</t>
+          <t>Regional Shenandoah Valley cancel wave; Public backlash</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Salem Mayor Dominick Pangallo and Police Chief Lucas Miller said the city would not renew Flock and would remove installed ALPRs over insufficient data protections, while seeking systems that better retain local control, a cancel-then-replace risk pattern.</t>
+          <t>Elkton ended its Flock contract the week before Harrisonburg’s July 29, 2026 cancel, per regional coverage of the Shenandoah Valley exit wave (alongside earlier Staunton / Charlottesville exits).</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>https://www.boston.com/news/local-news/2026/07/26/salem-joins-list-of-mass-communities-to-reject-surveillance-company-over-data-concerns/</t>
+          <t>https://www.dnronline.com/news/public_safety/harrisonburg-city-council-votes-to-cancel-flock-camera-contract/article_e96103ea-5a30-5d31-9d9c-3198e8ae5c9e.html</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.wcvb.com/article/flock-camera-contract-ending-salem-ma-july-24/73258537</t>
+          <t>https://www.29news.com/2026/07/29/harrisonburg-city-council-votes-end-contract-with-flock-safety/</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3383,38 +3379,35 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>City indicated intent to replace with another ALPR vendor retaining local data control.</t>
+          <t>Camera count and exact council vote date not detailed in Harrisonburg-focused coverage.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAN-2026-047</t>
+          <t>CAN-2026-046</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Monroe County</t>
+          <t>Salem</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Terminated</t>
+          <t>Non-renewal</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="F48" t="n">
-        <v>6</v>
+          <t>2026-07</t>
+        </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3428,22 +3421,22 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Privacy / mass-surveillance concerns; Outside and federal access risk; Physical removal emphasis</t>
+          <t>Data ownership / local-control concerns; Seeking replacement vendor</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Monroe County Commissioners voted to cancel the Flock contract (~6 cameras), citing privacy and mass-surveillance concerns and risk that plate/location data could be accessed by outside or federal agencies. Coverage notes Bloomington also ending its Flock contract; officials emphasized cameras must come down, not only contracts ending. CBS4 Indy / WIBC / WBIW July 28, 2026.</t>
+          <t>Salem Mayor Dominick Pangallo and Police Chief Lucas Miller said the city would not renew Flock and would remove installed ALPRs over insufficient data protections, while seeking systems that better retain local control, a cancel-then-replace risk pattern.</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>https://cbs4indy.com/news/monroe-county-ditches-flock-cameras-citing-privacy-concerns/</t>
+          <t>https://www.boston.com/news/local-news/2026/07/26/salem-joins-list-of-mass-communities-to-reject-surveillance-company-over-data-concerns/</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://wibc.com/893233/monroe-county-ditches-flock-cameras-over-privacy-concerns/</t>
+          <t>https://www.wcvb.com/article/flock-camera-contract-ending-salem-ma-july-24/73258537</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3453,24 +3446,24 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>YouTube: https://www.youtube.com/watch?v=eguU9gQfZ54 (CBS4 Indy). Bloomington city exit tracked separately (CAN-2026-017).</t>
+          <t>City indicated intent to replace with another ALPR vendor retaining local data control.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAN-2026-048</t>
+          <t>CAN-2026-047</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Stoughton</t>
+          <t>Monroe County</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>WI</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3484,7 +3477,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -3498,22 +3491,22 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Public backlash; Privacy concerns; Early buyout of two-year contract</t>
+          <t>Privacy / mass-surveillance concerns; Outside and federal access risk; Physical removal emphasis</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Stoughton City Council unanimously voted July 28, 2026 to terminate Flock after months of resident opposition. Five cameras (four ALPR + one live feed); ~$12,500 remaining buyout on a two-year/$25,000 contract; removal and data deletion directed; commitment not to swap to similar tech without 30 days’ notice and public input. Seventh Dane County entity ending Flock per local reporting.</t>
+          <t>Monroe County Commissioners voted to cancel the Flock contract (~6 cameras), citing privacy and mass-surveillance concerns and risk that plate/location data could be accessed by outside or federal agencies. Coverage notes Bloomington also ending its Flock contract; officials emphasized cameras must come down, not only contracts ending. CBS4 Indy / WIBC / WBIW July 28, 2026.</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>https://www.wmtv15news.com/2026/07/29/stoughton-city-council-unanimously-votes-terminate-agreement-with-flock-safety/</t>
+          <t>https://cbs4indy.com/news/monroe-county-ditches-flock-cameras-citing-privacy-concerns/</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.channel3000.com/news/stoughton-council-members-vote-to-terminate-flock-contract/article_cd05b0a6-881a-48ef-b0d2-bddb24d2a343.html</t>
+          <t>https://wibc.com/893233/monroe-county-ditches-flock-cameras-over-privacy-concerns/</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3523,24 +3516,24 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>YouTube: https://www.youtube.com/watch?v=4NtGB6BMvFU (WKOW 27). WKOW video page: https://www.wkow.com/video/stoughton-votes-to-remove-flock-cameras/video_5cb9e98e-a618-5f0b-bff7-71342db8f8c6.html</t>
+          <t>YouTube: https://www.youtube.com/watch?v=eguU9gQfZ54 (CBS4 Indy). Bloomington city exit tracked separately (CAN-2026-017).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAN-2026-049</t>
+          <t>CAN-2026-048</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>South Kingstown</t>
+          <t>Stoughton</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>WI</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3550,11 +3543,11 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -3568,22 +3561,22 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Public backlash; Privacy concerns; ACLU of RI advocacy letter; Misuse/federal-access fears</t>
+          <t>Public backlash; Privacy concerns; Early buyout of two-year contract</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>South Kingstown Town Council voted unanimously (5-0) on July 27, 2026 to terminate Flock and remove cameras ASAP after hundreds of resident emails and an ACLU of Rhode Island letter. Contract ~$30,300/year; ~6-7 cameras active since Feb 2026. Seeking partial refund. State Police Flock on state roads may remain nearby.</t>
+          <t>Stoughton City Council unanimously voted July 28, 2026 to terminate Flock after months of resident opposition. Five cameras (four ALPR + one live feed); ~$12,500 remaining buyout on a two-year/$25,000 contract; removal and data deletion directed; commitment not to swap to similar tech without 30 days’ notice and public input. Seventh Dane County entity ending Flock per local reporting.</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>https://www.wpri.com/news/local-news/south-county/south-kingstown-to-stop-using-automated-license-plate-readers/</t>
+          <t>https://www.wmtv15news.com/2026/07/29/stoughton-city-council-unanimously-votes-terminate-agreement-with-flock-safety/</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://turnto10.com/news/local/south-kingstown-ends-partnership-with-flock-cameras-july-28-2026</t>
+          <t>https://www.channel3000.com/news/stoughton-council-members-vote-to-terminate-flock-contract/article_cd05b0a6-881a-48ef-b0d2-bddb24d2a343.html</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -3593,24 +3586,24 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>YouTube WPRI https://www.youtube.com/watch?v=5a4l65Jen3E and WJAR https://www.youtube.com/watch?v=9RRqBtry1CU cover the same South Kingstown cancel. ACLU RI: https://www.riaclu.org/news/south-kingstown-cancels-flock-safety-contract-after-community-advocacy-aclu-letter/</t>
+          <t>YouTube: https://www.youtube.com/watch?v=4NtGB6BMvFU (WKOW 27). WKOW video page: https://www.wkow.com/video/stoughton-votes-to-remove-flock-cameras/video_5cb9e98e-a618-5f0b-bff7-71342db8f8c6.html</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAN-2026-050</t>
+          <t>CAN-2026-049</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Littleton</t>
+          <t>South Kingstown</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3620,11 +3613,11 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -3638,22 +3631,22 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Vendor trust failure; Unauthorized reactivation without notice; Privacy review</t>
+          <t>Public backlash; Privacy concerns; ACLU of RI advocacy letter; Misuse/federal-access fears</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>After a May 2026 Select Board order powered down six Flock cameras for policy review, police found on July 30 that Flock had reactivated five of six cameras on public ways without notifying the town. Select Board cut power, ordered contract termination, and directed removal of all six cameras.</t>
+          <t>South Kingstown Town Council voted unanimously (5-0) on July 27, 2026 to terminate Flock and remove cameras ASAP after hundreds of resident emails and an ACLU of Rhode Island letter. Contract ~$30,300/year; ~6-7 cameras active since Feb 2026. Seeking partial refund. State Police Flock on state roads may remain nearby.</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>https://shrewsburypost.com/2026/08/02/littleton-cancels-flock-safety-contract-after-cameras-reactivated-without-notice/</t>
+          <t>https://www.wpri.com/news/local-news/south-county/south-kingstown-to-stop-using-automated-license-plate-readers/</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.lowellsun.com/2026/07/31/littleton-claims-flock-reactivated-its-cameras-without-notifying-the-town/</t>
+          <t>https://turnto10.com/news/local/south-kingstown-ends-partnership-with-flock-cameras-july-28-2026</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -3663,24 +3656,24 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>Power cut immediately; physical removal ordered for all six public-way units.</t>
+          <t>YouTube WPRI https://www.youtube.com/watch?v=5a4l65Jen3E and WJAR https://www.youtube.com/watch?v=9RRqBtry1CU cover the same South Kingstown cancel. ACLU RI: https://www.riaclu.org/news/south-kingstown-cancels-flock-safety-contract-after-community-advocacy-aclu-letter/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAN-2026-051</t>
+          <t>CAN-2026-050</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Narragansett</t>
+          <t>Littleton</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>RI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3690,11 +3683,11 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -3708,22 +3701,22 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Public backlash; Early-exit accepted; Low local crime cited; RI cancel wave</t>
+          <t>Vendor trust failure; Unauthorized reactivation without notice; Privacy review</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Narragansett Town Council voted unanimously August 3, 2026 to terminate Flock early and accept early-exit penalties. Agreement had been set to run into 2027; about four cameras (one stolen). Came one week after South Kingstown’s cancel. Boston Globe notes ~$12,600 initial / ~$12,000 yearly from forfeiture funds.</t>
+          <t>After a May 2026 Select Board order powered down six Flock cameras for policy review, police found on July 30 that Flock had reactivated five of six cameras on public ways without notifying the town. Select Board cut power, ordered contract termination, and directed removal of all six cameras.</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>https://www.wpri.com/news/local-news/south-county/narragansett-to-stop-using-automated-license-plate-readers/</t>
+          <t>https://shrewsburypost.com/2026/08/02/littleton-cancels-flock-safety-contract-after-cameras-reactivated-without-notice/</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.bostonglobe.com/2026/08/04/metro/narragansett-town-council-ends-flock-safety-contract-ri/</t>
+          <t>https://www.lowellsun.com/2026/07/31/littleton-claims-flock-reactivated-its-cameras-without-notifying-the-town/</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -3733,38 +3726,38 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>WJAR Aug 4 confirm; GoLocalProv covers RI wave after South Kingstown.</t>
+          <t>Power cut immediately; physical removal ordered for all six public-way units.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAN-2026-052</t>
+          <t>CAN-2026-051</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Narragansett</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>RI</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Paused</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -3778,22 +3771,22 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Public backlash; Privacy / nationwide sharing concerns; Contract-language amendment</t>
+          <t>Public backlash; Early-exit accepted; Low local crime cited; RI cancel wave</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Oklahoma City Council deferred an August 4, 2026 vote on a ~$270,000 Flock renewal (~90 cameras through June 30, 2027) so staff could amend agreement language. Journal Record says the system had been running without a valid contract since July 1; item expected back about August 18. Not a cancel—a delayed renewal under public pressure.</t>
+          <t>Narragansett Town Council voted unanimously August 3, 2026 to terminate Flock early and accept early-exit penalties. Agreement had been set to run into 2027; about four cameras (one stolen). Came one week after South Kingstown’s cancel. Boston Globe notes ~$12,600 initial / ~$12,000 yearly from forfeiture funds.</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>https://journalrecord.com/2026/08/04/oklahoma-city-delays-flock-camera-contract-resident-concerns/</t>
+          <t>https://www.wpri.com/news/local-news/south-county/narragansett-to-stop-using-automated-license-plate-readers/</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.oklahoman.com/story/news/local/oklahoma-city/2026/08/03/okc-stalls-vote-flock-cameras-renewal/91159028007/</t>
+          <t>https://www.bostonglobe.com/2026/08/04/metro/narragansett-town-council-ends-flock-safety-contract-ri/</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -3803,38 +3796,38 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>Cameras reportedly still active pending Aug 18 return; not a termination.</t>
+          <t>WJAR Aug 4 confirm; GoLocalProv covers RI wave after South Kingstown.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAN-2026-053</t>
+          <t>CAN-2026-052</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Ord</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Terminated</t>
+          <t>Paused</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -3848,22 +3841,22 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Public backlash; Privacy concerns; First Nebraska municipal reject</t>
+          <t>Public backlash; Privacy / nationwide sharing concerns; Contract-language amendment</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Ord City Council voted 5-0 on August 3, 2026 to begin removing two Flock cameras, described as Nebraska’s first outright municipal reject. Cameras were installed under a Valley County / Region 26 emergency-management grant and were still operating after the city vote pending county / Region 26 follow-up (board discussion aimed around Aug. 11).</t>
+          <t>Oklahoma City Council deferred an August 4, 2026 vote on a ~$270,000 Flock renewal (~90 cameras through June 30, 2027) so staff could amend agreement language. Journal Record says the system had been running without a valid contract since July 1; item expected back about August 18. Not a cancel—a delayed renewal under public pressure.</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>https://www.wowt.com/2026/08/04/city-ord-votes-unanimously-remove-its-flock-cameras-first-nebraska/</t>
+          <t>https://journalrecord.com/2026/08/04/oklahoma-city-delays-flock-camera-contract-resident-concerns/</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://kgfw.com/2026/08/04/ord-city-council-votes-to-remove-flock-cameras/</t>
+          <t>https://www.oklahoman.com/story/news/local/oklahoma-city/2026/08/03/okc-stalls-vote-flock-cameras-renewal/91159028007/</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -3873,24 +3866,24 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>County ownership / Region 26 grant means city vote alone may not power cameras down; removal coordination ongoing as of Aug. 4 reporting.</t>
+          <t>Cameras reportedly still active pending Aug 18 return; not a termination.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAN-2026-054</t>
+          <t>CAN-2026-053</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Stanford University</t>
+          <t>Ord</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3900,8 +3893,11 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
-        </is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>2</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -3915,22 +3911,22 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Third-party / network access risk; Campus privacy backlash; Vendor swap</t>
+          <t>Public backlash; Privacy concerns; First Nebraska municipal reject</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Stanford University announced it ended its Flock Safety agreement and is replacing campus entrance ALPR with Genetec Cloudrunner: short cloud hold, then university-controlled storage with no third-party network access built into the architecture (Palo Alto Online citing Stanford Report, Aug. 4, 2026). Note: swapping vendors is not ending campus ALPR.</t>
+          <t>Ord City Council voted 5-0 on August 3, 2026 to begin removing two Flock cameras, described as Nebraska’s first outright municipal reject. Cameras were installed under a Valley County / Region 26 emergency-management grant and were still operating after the city vote pending county / Region 26 follow-up (board discussion aimed around Aug. 11).</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>https://www.paloaltoonline.com/news/2026/08/04/stanford-drops-flock-cameras-amid-national-backlash/</t>
+          <t>https://www.wowt.com/2026/08/04/city-ord-votes-unanimously-remove-its-flock-cameras-first-nebraska/</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://news.stanford.edu/stories/2024/09/stanford-to-install-license-plate-cameras-at-campus-entrances</t>
+          <t>https://kgfw.com/2026/08/04/ord-city-council-votes-to-remove-flock-cameras/</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -3940,34 +3936,34 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>Campus ALPR continues under Genetec; Flock exit is a network-isolation choice, not a plate-scanner ban.</t>
+          <t>County ownership / Region 26 grant means city vote alone may not power cameras down; removal coordination ongoing as of Aug. 4 reporting.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAN-2026-055</t>
+          <t>CAN-2026-054</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Pinal County</t>
+          <t>Stanford University</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Non-renewal</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3982,22 +3978,22 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Fourth Amendment concerns; Sheriff non-renewal; Privacy / mass-surveillance risk</t>
+          <t>Third-party / network access risk; Campus privacy backlash; Vendor swap</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Pinal County Sheriff Ross Teeple told the Board of Supervisors on August 5, 2026 he will not renew the sheriff’s office Flock Safety contract when it expires at the end of September, citing serious Fourth Amendment concerns about the technology whether or not the county uses every feature. Teeple had defended the cameras at a 2025 town hall. Cities and towns inside the county that run their own Flock programs are not bound by the sheriff’s decision. Decommissioning was expected as the contract lapses.</t>
+          <t>Stanford University announced it ended its Flock Safety agreement and is replacing campus entrance ALPR with Genetec Cloudrunner: short cloud hold, then university-controlled storage with no third-party network access built into the architecture (Palo Alto Online citing Stanford Report, Aug. 4, 2026). Note: swapping vendors is not ending campus ALPR.</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>https://www.azfamily.com/2026/08/06/pinal-county-chooses-not-renew-flock-camera-contract/</t>
+          <t>https://www.paloaltoonline.com/news/2026/08/04/stanford-drops-flock-cameras-amid-national-backlash/</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.fox10phoenix.com/news/pinal-county-sheriff-pulls-plug-flock-license-plate-cameras-he-once-praised</t>
+          <t>https://news.stanford.edu/stories/2024/09/stanford-to-install-license-plate-cameras-at-campus-entrances</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -4007,19 +4003,19 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>Sheriff’s office cameras only; municipal Flock programs inside Pinal County may continue. Hardware removal timing after September lapse still TBD. Official PCSO Facebook reel: https://www.facebook.com/reel/3622783047870589</t>
+          <t>Campus ALPR continues under Genetec; Flock exit is a network-isolation choice, not a plate-scanner ban.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAN-2026-056</t>
+          <t>CAN-2026-055</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>South Tucson</t>
+          <t>Pinal County</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -4029,17 +4025,17 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Terminated</t>
+          <t>Non-renewal</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -4049,44 +4045,44 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Public backlash; Privacy / mass-surveillance concerns; Data-sharing concerns</t>
+          <t>Fourth Amendment concerns; Sheriff non-renewal; Privacy / mass-surveillance risk</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>South Tucson City Council voted February 17, 2026 to cancel its Flock Safety contract after months of resident opposition organized in part by Deflock Tucson, making South Tucson the third Arizona city in that reporting wave after Flagstaff and Sedona. Officials later explored alternative surveillance options while police said losing the tool affected investigations.</t>
+          <t>Pinal County Sheriff Ross Teeple told the Board of Supervisors on August 5, 2026 he will not renew the sheriff’s office Flock Safety contract when it expires at the end of September, citing serious Fourth Amendment concerns about the technology whether or not the county uses every feature. Teeple had defended the cameras at a 2025 town hall. Cities and towns inside the county that run their own Flock programs are not bound by the sheriff’s decision. Decommissioning was expected as the contract lapses.</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>https://www.tucsonspotlight.org/south-tucson-ends-flock-camera-contract/</t>
+          <t>https://www.azfamily.com/2026/08/06/pinal-county-chooses-not-renew-flock-camera-contract/</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.kgun9.com/news/community-inspired-journalism/south-tucson/south-tucson-ends-flock-camera-contract-city-now-searching-for-alternatives</t>
+          <t>https://www.fox10phoenix.com/news/pinal-county-sheriff-pulls-plug-flock-license-plate-cameras-he-once-praised</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Verified local/primary</t>
+          <t>Verified major press</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>Council explored replacement surveillance vendors after the Flock exit.</t>
+          <t>Sheriff’s office cameras only; municipal Flock programs inside Pinal County may continue. Hardware removal timing after September lapse still TBD. Official PCSO Facebook reel: https://www.facebook.com/reel/3622783047870589</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAN-2026-057</t>
+          <t>CAN-2026-056</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Sierra Vista</t>
+          <t>South Tucson</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -4101,11 +4097,8 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>16</v>
+          <t>2026-02-17</t>
+        </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -4119,17 +4112,22 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Public backlash; Data ownership / AI training concerns; Vendor swap planned</t>
+          <t>Public backlash; Privacy / mass-surveillance concerns; Data-sharing concerns</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Sierra Vista City Council directed staff in a February 24, 2026 work session to end the Flock contract (30-day notice); city officials said the agreement was officially terminated April 2, 2026. About 16 grant-funded plate readers had been purchased for police. Residents and Cochise County Supervisor Frank Antenori raised concerns about Flock owning image rights and AI use. Cameras remained mounted but offline pending Flock removal; the city planned to seek another ALPR vendor with the same grant funds.</t>
+          <t>South Tucson City Council voted February 17, 2026 to cancel its Flock Safety contract after months of resident opposition organized in part by Deflock Tucson, making South Tucson the third Arizona city in that reporting wave after Flagstaff and Sedona. Officials later explored alternative surveillance options while police said losing the tool affected investigations.</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>https://www.kgun9.com/news/community-inspired-journalism/cochise-county/sierra-vista-ends-contract-with-flock</t>
+          <t>https://www.tucsonspotlight.org/south-tucson-ends-flock-camera-contract/</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>https://www.kgun9.com/news/community-inspired-journalism/south-tucson/south-tucson-ends-flock-camera-contract-city-now-searching-for-alternatives</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -4139,24 +4137,24 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>Hardware still up but not operational pending vendor removal; city shopping replacement ALPR.</t>
+          <t>Council explored replacement surveillance vendors after the Flock exit.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAN-2026-058</t>
+          <t>CAN-2026-057</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Albany</t>
+          <t>Sierra Vista</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>OR</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4166,15 +4164,15 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4184,64 +4182,62 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Public backlash; Federal access / privacy concerns; Early termination fee</t>
+          <t>Public backlash; Data ownership / AI training concerns; Vendor swap planned</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Albany City Council voted 4-2 on May 27–28, 2026 to end its Flock Safety contract after earlier suspending the city’s single active downtown camera in February over federal-access concerns. The camera was stolen after power-down. Formal termination was effective June 29; early exit cost about $7,000 per city manager reporting. Plans for three additional cameras were dropped.</t>
+          <t>Sierra Vista City Council directed staff in a February 24, 2026 work session to end the Flock contract (30-day notice); city officials said the agreement was officially terminated April 2, 2026. About 16 grant-funded plate readers had been purchased for police. Residents and Cochise County Supervisor Frank Antenori raised concerns about Flock owning image rights and AI use. Cameras remained mounted but offline pending Flock removal; the city planned to seek another ALPR vendor with the same grant funds.</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>https://www.klcc.org/politics-government/2026-05-28/albany-city-council-decides-against-reactivating-flock-camera</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>https://www.govtech.com/public-safety/flock-safety-suspension-costs-oregon-city-7-000</t>
+          <t>https://www.kgun9.com/news/community-inspired-journalism/cochise-county/sierra-vista-ends-contract-with-flock</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Verified major press</t>
+          <t>Verified local/primary</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>Only one camera had been deployed of four purchased; stolen after February suspension.</t>
+          <t>Hardware still up but not operational pending vendor removal; city shopping replacement ALPR.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAN-2026-059</t>
+          <t>CAN-2026-058</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Chandler</t>
+          <t>Albany</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Paused</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-08</t>
-        </is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>1</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4251,22 +4247,22 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Public backlash; Renewal delay; Privacy / ordinance campaign</t>
+          <t>Public backlash; Federal access / privacy concerns; Early termination fee</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Chandler City Council delayed a decision on renewing its about $153,000 Flock Safety contract until its August 13, 2026 meeting amid resident opposition organized by East Valley Unite and related advocacy. FOX 10 / AZFamily reporting on the Pinal County non-renewal wave noted Chandler’s delay alongside Flagstaff, Sedona, and South Tucson exits. Not a cancel—a delayed renewal under public pressure.</t>
+          <t>Albany City Council voted 4-2 on May 27–28, 2026 to end its Flock Safety contract after earlier suspending the city’s single active downtown camera in February over federal-access concerns. The camera was stolen after power-down. Formal termination was effective June 29; early exit cost about $7,000 per city manager reporting. Plans for three additional cameras were dropped.</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>https://www.fox10phoenix.com/news/pinal-county-sheriff-pulls-plug-flock-license-plate-cameras-he-once-praised</t>
+          <t>https://www.klcc.org/politics-government/2026-05-28/albany-city-council-decides-against-reactivating-flock-camera</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.azcentral.com/story/news/politics/arizona/2026/07/08/flock-cameras-raise-privacy-safety-concerns-in-arizona/90841857007/</t>
+          <t>https://www.govtech.com/public-safety/flock-safety-suspension-costs-oregon-city-7-000</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -4276,34 +4272,34 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>Cameras still in use pending Aug. 13 renewal vote; not a termination.</t>
+          <t>Only one camera had been deployed of four purchased; stolen after February suspension.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAN-2026-060</t>
+          <t>CAN-2026-059</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Sumter County</t>
+          <t>Chandler</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Suspended</t>
+          <t>Paused</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -4313,27 +4309,27 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Officer database / ALPR misuse; Internal audit; Agency integrity response</t>
+          <t>Public backlash; Renewal delay; Privacy / ordinance campaign</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Sumter County Sheriff Patrick Breeden suspended the Sheriff’s Office use of Flock after an internal audit flagged Detective Brandy Almany’s alleged personal-use searches of Flock ALPR, Florida’s DAVID, and CCIS involving her husband’s ex-wife. Almany was arrested and terminated (July 23, 2026). Breeden ordered a complete internal audit of agency databases while Flock remains suspended.</t>
+          <t>Chandler City Council delayed a decision on renewing its about $153,000 Flock Safety contract until its August 13, 2026 meeting amid resident opposition organized by East Valley Unite and related advocacy. FOX 10 / AZFamily reporting on the Pinal County non-renewal wave noted Chandler’s delay alongside Flagstaff, Sedona, and South Tucson exits. Not a cancel—a delayed renewal under public pressure.</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>https://www.wftv.com/news/local/sumter-detective-fired-arrested-using-police-cameras-spy-husbands-ex-wife/O2ZIHFAP4FC7VINFSGNDGPU6DI/</t>
+          <t>https://www.fox10phoenix.com/news/pinal-county-sheriff-pulls-plug-flock-license-plate-cameras-he-once-praised</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.wesh.com/article/sumter-detective-arrested-database-misuse/73251430</t>
+          <t>https://www.azcentral.com/story/news/politics/arizona/2026/07/08/flock-cameras-raise-privacy-safety-concerns-in-arizona/90841857007/</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -4343,74 +4339,277 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>Temporary suspension pending complete internal audit; agency had not announced when or whether cameras would return as of July 24, 2026 reporting. Related misuse row: FLK-2026-020.</t>
+          <t>Cameras still in use pending Aug. 13 renewal vote; not a termination.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>CAN-2026-060</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Sumter County</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Suspended</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Officer database / ALPR misuse; Internal audit; Agency integrity response</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Sumter County Sheriff Patrick Breeden suspended the Sheriff’s Office use of Flock after an internal audit flagged Detective Brandy Almany’s alleged personal-use searches of Flock ALPR, Florida’s DAVID, and CCIS involving her husband’s ex-wife. Almany was arrested and terminated (July 23, 2026). Breeden ordered a complete internal audit of agency databases while Flock remains suspended.</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>https://www.wftv.com/news/local/sumter-detective-fired-arrested-using-police-cameras-spy-husbands-ex-wife/O2ZIHFAP4FC7VINFSGNDGPU6DI/</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>https://www.wesh.com/article/sumter-detective-arrested-database-misuse/73251430</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Temporary suspension pending complete internal audit; agency had not announced when or whether cameras would return as of July 24, 2026 reporting. Related misuse row: FLK-2026-020.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>CAN-2026-061</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Leon County</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>Pre-install cancel</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
         <is>
           <t>Public backlash; Privacy / surveillance concerns; Regional grant reject</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>Leon County Commission on July 14, 2026 unanimously stripped about $440,000 in regional public-safety grant funding that would have expanded Flock ALPRs in neighboring Wakulla, Jefferson, Liberty, and Taylor counties (pass-through via Leon County Sheriff’s Office). Commissioners approved other grant items, directed a September workshop on county authority to regulate or ban ALPRs locally, after packed public comment opposing surveillance expansion.</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t>https://www.tallahassee.com/story/news/local/2026/07/16/leon-county-rejects-grants-for-flock-license-plate-readers/90930124007/</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr">
+      <c r="L63" t="inlineStr">
         <is>
           <t>https://news.wfsu.org/wfsu-local-news/2026-07-14/leon-commissioners-pass-data-center-moratorium-block-flock-camera-grant-funding</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
+      <c r="M63" t="inlineStr">
         <is>
           <t>Verified major press</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr">
+      <c r="N63" t="inlineStr">
         <is>
           <t>Rejects regional expansion grant funding, not removal of existing Leon County cameras; September 2026 authority/workshop follow-up pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>CAN-2026-062</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Syracuse</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Terminated</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>13</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Data-sharing controversies; Public backlash; Vendor swap (Axon)</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>After data-sharing controversies, Syracuse Common Council moved to end Flock on city streets and approved a multi-year Axon plate-reader contract. By mid-July 2026, Flock confirmed its 13 city-approved readers were removed from city property. Axon cameras were expected afterward: a vendor swap, not an end to mass plate scanning. Separate university / private Flock installs can remain.</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>https://spectrumlocalnews.com/nys/central-ny/politics/2026/07/23/all-flock-cameras-in-syracuse-have-been-removed</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>https://centralcurrent.org/flock-safety-removes-its-license-plate-readers-finalizing-eight-month-breakup-with-city-of-syracuse/</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>City property Flock removed; Axon replacement approved. Private / university Flock units may remain. Not a ban on ALPR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>CAN-2026-063</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Grand Chute</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Terminated</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>23</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Public backlash; Privacy concerns; Vendor swap (Axon)</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Grand Chute’s board canceled its Flock contract and signed an Axon camera agreement the same night. Reporting says about 23 cameras stay in place for a swap targeted around September 1: another Flock-to-Axon vendor swap, not an end to plate scanning.</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>https://fox11online.com/news/local/grand-chute-cancels-flock-contract-signs-camera-agreement-with-new-company-axon-safety-privacy</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Verified major press</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Flock exit with same-night Axon replacement; cameras remain for swap. Not a ban on ALPR.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Aug. 7–8 Flock stories: Chandler cancel, Savannah firings, Royston, Elk Grove audit.
Sync misuse and cancel dossiers (56 / 53 exits) with matching site tallies and sources.
</commit_message>
<xml_diff>
--- a/docs/Flock_Municipal_Cancellations_Database.xlsx
+++ b/docs/Flock_Municipal_Cancellations_Database.xlsx
@@ -4294,17 +4294,20 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Paused</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-08</t>
-        </is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>40</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -4314,24 +4317,24 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Public backlash; Renewal delay; Privacy / ordinance campaign</t>
+          <t>Officer / employee ALPR misuse anomaly; Public backlash; Administrative non-renewal</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Chandler City Council delayed a decision on renewing its about $153,000 Flock Safety contract until its August 13, 2026 meeting amid resident opposition organized by East Valley Unite and related advocacy. FOX 10 / AZFamily reporting on the Pinal County non-renewal wave noted Chandler’s delay alongside Flagstaff, Sedona, and South Tucson exits. Not a cancel—a delayed renewal under public pressure.</t>
+          <t>Chandler ended its about $153,000 Flock Safety contract on August 7, 2026 after a routine audit found an unexplained anomaly in system use on August 6. Police Chief Bryan Chapman said an internal investigation would determine whether Flock was used inappropriately. The city had delayed a renewal vote to August 13 amid resident opposition; spokespeople said not renewing can be an administrative decision without that council vote. About 40 fixed cameras; access restricted pending removal. Largest Arizona city to drop Flock in contemporaneous coverage. Related misuse row: FLK-2026-034.</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
+          <t>https://www.azcentral.com/story/news/local/chandler-breaking/2026/08/07/chandler-arizona-discontinues-flock-cameras/91218403007/</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
           <t>https://www.fox10phoenix.com/news/pinal-county-sheriff-pulls-plug-flock-license-plate-cameras-he-once-praised</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>https://www.azcentral.com/story/news/politics/arizona/2026/07/08/flock-cameras-raise-privacy-safety-concerns-in-arizona/90841857007/</t>
-        </is>
-      </c>
       <c r="M61" t="inlineStr">
         <is>
           <t>Verified major press</t>
@@ -4339,7 +4342,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>Cameras still in use pending Aug. 13 renewal vote; not a termination.</t>
+          <t>Cameras still mounted pending Flock removal coordination; department cut system access. Safeguards review before any future ALPR discussion. Misuse probe open.</t>
         </is>
       </c>
     </row>

</xml_diff>